<commit_message>
Add SOH report for 2026-10-13
</commit_message>
<xml_diff>
--- a/reports/SOH_12_10_2026.xlsx
+++ b/reports/SOH_12_10_2026.xlsx
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>149</v>
+        <v>122</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1049</v>
+        <v>949</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>2800</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1107</v>
+        <v>1101</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>481</v>
+        <v>471</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>10500</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1023</v>
+        <v>1014</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E46" s="3" t="n">
         <v>21000</v>
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>81000</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>881</v>
+        <v>815</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>3000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>663</v>
+        <v>603</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>3000</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>725</v>
+        <v>676</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E103" s="3" t="n">
         <v>4708</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="E104" s="3" t="n">
         <v>4708</v>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E106" s="3" t="n">
         <v>12500</v>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E108" s="3" t="n">
         <v>1</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2746</v>
+        <v>2734</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>3876</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2150</v>
+        <v>2120</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>4743</v>
+        <v>4730</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>133</v>
+        <v>85</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4685,7 +4685,7 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E152" s="3" t="n">
         <v>1</v>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="E157" s="3" t="n">
         <v>1</v>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E168" s="3" t="n">
         <v>1</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="E174" s="3" t="n">
         <v>13500</v>
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E182" s="3" t="n">
         <v>1</v>
@@ -5724,23 +5724,23 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>API064</t>
+          <t>API019</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>AWB Promotional Items AIWIBI T-shirt (blue) S</t>
+          <t>AWB Promotional Items Baby Infltable Mold with LOGO</t>
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E191" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>PROMOTION</t>
+          <t>AIWIBI</t>
         </is>
       </c>
     </row>
@@ -5752,12 +5752,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>API016</t>
+          <t>API007</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>AWB Promotional Items AIWIBI T-shirt (blue) XXL</t>
+          <t>AWB Promotional Items Baby Model</t>
         </is>
       </c>
       <c r="D192" s="2" t="n">
@@ -5780,16 +5780,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>API019</t>
+          <t>API016</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>AWB Promotional Items Baby Infltable Mold with LOGO</t>
+          <t>AWB Promotional Items AIWIBI T-shirt (blue) XXL</t>
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E193" s="3" t="n">
         <v>0</v>
@@ -5803,24 +5803,24 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9309000257638</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>API007</t>
+          <t>API026</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>AWB Promotional Items Baby Model</t>
+          <t>AWB Promotional Items Baby Set Regular</t>
         </is>
       </c>
       <c r="D194" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E194" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F194" t="inlineStr">
         <is>
@@ -5831,28 +5831,28 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>9309000257638</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>API026</t>
+          <t>API064</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>AWB Promotional Items Baby Set Regular</t>
+          <t>AWB Promotional Items AIWIBI T-shirt (blue) S</t>
         </is>
       </c>
       <c r="D195" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E195" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>AIWIBI</t>
+          <t>PROMOTION</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -7441,7 +7441,7 @@
         </is>
       </c>
       <c r="D254" s="2" t="n">
-        <v>854</v>
+        <v>842</v>
       </c>
       <c r="E254" s="3" t="n">
         <v>11491</v>
@@ -7833,7 +7833,7 @@
         </is>
       </c>
       <c r="D268" s="2" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E268" s="3" t="n">
         <v>13890</v>
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="D274" s="2" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="E274" s="3" t="n">
         <v>3954</v>
@@ -8981,7 +8981,7 @@
         </is>
       </c>
       <c r="D309" s="2" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E309" s="3" t="n">
         <v>26979</v>
@@ -9037,7 +9037,7 @@
         </is>
       </c>
       <c r="D311" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E311" s="3" t="n">
         <v>9760</v>
@@ -9177,7 +9177,7 @@
         </is>
       </c>
       <c r="D316" s="2" t="n">
-        <v>473</v>
+        <v>461</v>
       </c>
       <c r="E316" s="3" t="n">
         <v>39894</v>
@@ -9289,7 +9289,7 @@
         </is>
       </c>
       <c r="D320" s="2" t="n">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="E320" s="3" t="n">
         <v>16171</v>
@@ -9766,7 +9766,7 @@
         </is>
       </c>
       <c r="D337" s="2" t="n">
-        <v>634</v>
+        <v>610</v>
       </c>
       <c r="E337" s="3" t="n">
         <v>9872</v>
@@ -9906,7 +9906,7 @@
         </is>
       </c>
       <c r="D342" s="2" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E342" s="3" t="n">
         <v>6251</v>
@@ -11866,7 +11866,7 @@
         </is>
       </c>
       <c r="D412" s="2" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E412" s="3" t="n">
         <v>53004</v>
@@ -12734,7 +12734,7 @@
         </is>
       </c>
       <c r="D443" s="2" t="n">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="E443" s="3" t="n">
         <v>37709</v>
@@ -13042,7 +13042,7 @@
         </is>
       </c>
       <c r="D454" s="2" t="n">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E454" s="3" t="n">
         <v>15206</v>
@@ -13126,7 +13126,7 @@
         </is>
       </c>
       <c r="D457" s="2" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E457" s="3" t="n">
         <v>7235</v>
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="D459" s="2" t="n">
-        <v>581</v>
+        <v>569</v>
       </c>
       <c r="E459" s="3" t="n">
         <v>9544</v>
@@ -13266,7 +13266,7 @@
         </is>
       </c>
       <c r="D462" s="2" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E462" s="3" t="n">
         <v>14997</v>
@@ -13350,7 +13350,7 @@
         </is>
       </c>
       <c r="D465" s="2" t="n">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E465" s="3" t="n">
         <v>11864</v>
@@ -13882,7 +13882,7 @@
         </is>
       </c>
       <c r="D484" s="2" t="n">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="E484" s="3" t="n">
         <v>5942</v>
@@ -13938,7 +13938,7 @@
         </is>
       </c>
       <c r="D486" s="2" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E486" s="3" t="n">
         <v>23611</v>
@@ -14862,7 +14862,7 @@
         </is>
       </c>
       <c r="D519" s="2" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E519" s="3" t="n">
         <v>12900</v>
@@ -14974,7 +14974,7 @@
         </is>
       </c>
       <c r="D523" s="2" t="n">
-        <v>5110</v>
+        <v>5086</v>
       </c>
       <c r="E523" s="3" t="n">
         <v>10621</v>
@@ -15926,7 +15926,7 @@
         </is>
       </c>
       <c r="D557" s="2" t="n">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E557" s="3" t="n">
         <v>10491</v>
@@ -15954,7 +15954,7 @@
         </is>
       </c>
       <c r="D558" s="2" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E558" s="3" t="n">
         <v>30863</v>
@@ -16150,7 +16150,7 @@
         </is>
       </c>
       <c r="D565" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E565" s="3" t="n">
         <v>8752</v>
@@ -16486,7 +16486,7 @@
         </is>
       </c>
       <c r="D577" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E577" s="3" t="n">
         <v>7094</v>
@@ -16570,7 +16570,7 @@
         </is>
       </c>
       <c r="D580" s="2" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E580" s="3" t="n">
         <v>18839</v>
@@ -16626,7 +16626,7 @@
         </is>
       </c>
       <c r="D582" s="2" t="n">
-        <v>385</v>
+        <v>361</v>
       </c>
       <c r="E582" s="3" t="n">
         <v>11436</v>
@@ -16696,24 +16696,24 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>9333527144348</t>
+          <t>9333527779199</t>
         </is>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>BL0246</t>
+          <t>KS0000143</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>DRIP DRY HANGER ROUND 18PEG</t>
+          <t>DRY FOOD JAR WITH LID 2000ML</t>
         </is>
       </c>
       <c r="D585" s="2" t="n">
-        <v>154</v>
+        <v>21</v>
       </c>
       <c r="E585" s="3" t="n">
-        <v>17407</v>
+        <v>41764</v>
       </c>
       <c r="F585" t="inlineStr">
         <is>
@@ -16724,24 +16724,24 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>9333527779175</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>KS0000142</t>
+          <t>DT BAGS</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>DRY FOOD JAR WITH LID 1500ML</t>
+          <t>DT BAGS</t>
         </is>
       </c>
       <c r="D586" s="2" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E586" s="3" t="n">
-        <v>34055</v>
+        <v>0</v>
       </c>
       <c r="F586" t="inlineStr">
         <is>
@@ -16752,24 +16752,24 @@
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>9333527779199</t>
+          <t>9333527779175</t>
         </is>
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>KS0000143</t>
+          <t>KS0000142</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>DRY FOOD JAR WITH LID 2000ML</t>
+          <t>DRY FOOD JAR WITH LID 1500ML</t>
         </is>
       </c>
       <c r="D587" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E587" s="3" t="n">
-        <v>41764</v>
+        <v>34055</v>
       </c>
       <c r="F587" t="inlineStr">
         <is>
@@ -16780,24 +16780,24 @@
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4894158095249</t>
         </is>
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>DT BAGS</t>
+          <t>PA3915</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>DT BAGS</t>
+          <t>DURA CHEW - M/L</t>
         </is>
       </c>
       <c r="D588" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E588" s="3" t="n">
-        <v>0</v>
+        <v>34572</v>
       </c>
       <c r="F588" t="inlineStr">
         <is>
@@ -16808,24 +16808,24 @@
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>4894158095249</t>
+          <t>9333527144348</t>
         </is>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>PA3915</t>
+          <t>BL0246</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>DURA CHEW - M/L</t>
+          <t>DRIP DRY HANGER ROUND 18PEG</t>
         </is>
       </c>
       <c r="D589" s="2" t="n">
-        <v>10</v>
+        <v>154</v>
       </c>
       <c r="E589" s="3" t="n">
-        <v>34572</v>
+        <v>17407</v>
       </c>
       <c r="F589" t="inlineStr">
         <is>
@@ -16990,7 +16990,7 @@
         </is>
       </c>
       <c r="D595" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E595" s="3" t="n">
         <v>13111</v>
@@ -17607,7 +17607,7 @@
         </is>
       </c>
       <c r="D617" s="2" t="n">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="E617" s="3" t="n">
         <v>9776</v>
@@ -17971,7 +17971,7 @@
         </is>
       </c>
       <c r="D630" s="2" t="n">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="E630" s="3" t="n">
         <v>8711</v>
@@ -18615,7 +18615,7 @@
         </is>
       </c>
       <c r="D653" s="2" t="n">
-        <v>1080</v>
+        <v>1056</v>
       </c>
       <c r="E653" s="3" t="n">
         <v>11078</v>
@@ -20267,7 +20267,7 @@
         </is>
       </c>
       <c r="D712" s="2" t="n">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E712" s="3" t="n">
         <v>8443</v>
@@ -20547,7 +20547,7 @@
         </is>
       </c>
       <c r="D722" s="2" t="n">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E722" s="3" t="n">
         <v>4500</v>
@@ -20575,7 +20575,7 @@
         </is>
       </c>
       <c r="D723" s="2" t="n">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E723" s="3" t="n">
         <v>12992</v>
@@ -21191,7 +21191,7 @@
         </is>
       </c>
       <c r="D745" s="2" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E745" s="3" t="n">
         <v>9853</v>
@@ -21779,7 +21779,7 @@
         </is>
       </c>
       <c r="D766" s="2" t="n">
-        <v>683</v>
+        <v>647</v>
       </c>
       <c r="E766" s="3" t="n">
         <v>7465</v>
@@ -22703,7 +22703,7 @@
         </is>
       </c>
       <c r="D799" s="2" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E799" s="3" t="n">
         <v>5085</v>
@@ -23207,7 +23207,7 @@
         </is>
       </c>
       <c r="D817" s="2" t="n">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="E817" s="3" t="n">
         <v>16983</v>
@@ -23880,7 +23880,7 @@
         </is>
       </c>
       <c r="D841" s="2" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E841" s="3" t="n">
         <v>13122</v>
@@ -24665,7 +24665,7 @@
         </is>
       </c>
       <c r="D869" s="2" t="n">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E869" s="3" t="n">
         <v>11577</v>
@@ -24721,7 +24721,7 @@
         </is>
       </c>
       <c r="D871" s="2" t="n">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="E871" s="3" t="n">
         <v>14083</v>
@@ -28420,7 +28420,7 @@
         </is>
       </c>
       <c r="D1003" s="2" t="n">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="E1003" s="3" t="n">
         <v>11261</v>
@@ -28448,7 +28448,7 @@
         </is>
       </c>
       <c r="D1004" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E1004" s="3" t="n">
         <v>5499</v>
@@ -28756,7 +28756,7 @@
         </is>
       </c>
       <c r="D1015" s="2" t="n">
-        <v>685</v>
+        <v>661</v>
       </c>
       <c r="E1015" s="3" t="n">
         <v>2930</v>
@@ -29709,7 +29709,7 @@
         </is>
       </c>
       <c r="D1049" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E1049" s="3" t="n">
         <v>15896</v>
@@ -29905,7 +29905,7 @@
         </is>
       </c>
       <c r="D1056" s="2" t="n">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E1056" s="3" t="n">
         <v>19007</v>
@@ -30045,7 +30045,7 @@
         </is>
       </c>
       <c r="D1061" s="2" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="E1061" s="3" t="n">
         <v>7942</v>
@@ -30437,7 +30437,7 @@
         </is>
       </c>
       <c r="D1075" s="2" t="n">
-        <v>538</v>
+        <v>526</v>
       </c>
       <c r="E1075" s="3" t="n">
         <v>9226</v>
@@ -31305,7 +31305,7 @@
         </is>
       </c>
       <c r="D1106" s="2" t="n">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="E1106" s="3" t="n">
         <v>11372</v>
@@ -31543,24 +31543,24 @@
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
-          <t>9333527813497</t>
+          <t>9333527393784</t>
         </is>
       </c>
       <c r="B1115" t="inlineStr">
         <is>
-          <t>YA0000014</t>
+          <t>YA0011</t>
         </is>
       </c>
       <c r="C1115" t="inlineStr">
         <is>
-          <t>PARTY HEADBAND HAPPY BIRTHDAY 4 ASSORTED</t>
+          <t>PARTY KRAFT TAGS + STRING 20PK</t>
         </is>
       </c>
       <c r="D1115" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E1115" s="3" t="n">
-        <v>12425</v>
+        <v>2025</v>
       </c>
       <c r="F1115" t="inlineStr">
         <is>
@@ -31627,24 +31627,24 @@
     <row r="1118">
       <c r="A1118" t="inlineStr">
         <is>
-          <t>9333527393784</t>
+          <t>9333527107282</t>
         </is>
       </c>
       <c r="B1118" t="inlineStr">
         <is>
-          <t>YA0011</t>
+          <t>SC0102</t>
         </is>
       </c>
       <c r="C1118" t="inlineStr">
         <is>
-          <t>PARTY KRAFT TAGS + STRING 20PK</t>
+          <t>PARTY LOOT BAGS 16.5X23CM 10PK</t>
         </is>
       </c>
       <c r="D1118" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E1118" s="3" t="n">
-        <v>2025</v>
+        <v>2869</v>
       </c>
       <c r="F1118" t="inlineStr">
         <is>
@@ -31655,24 +31655,24 @@
     <row r="1119">
       <c r="A1119" t="inlineStr">
         <is>
-          <t>9333527107282</t>
+          <t>9333527813497</t>
         </is>
       </c>
       <c r="B1119" t="inlineStr">
         <is>
-          <t>SC0102</t>
+          <t>YA0000014</t>
         </is>
       </c>
       <c r="C1119" t="inlineStr">
         <is>
-          <t>PARTY LOOT BAGS 16.5X23CM 10PK</t>
+          <t>PARTY HEADBAND HAPPY BIRTHDAY 4 ASSORTED</t>
         </is>
       </c>
       <c r="D1119" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E1119" s="3" t="n">
-        <v>2869</v>
+        <v>12425</v>
       </c>
       <c r="F1119" t="inlineStr">
         <is>
@@ -32201,7 +32201,7 @@
         </is>
       </c>
       <c r="D1138" s="2" t="n">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="E1138" s="3" t="n">
         <v>4651</v>
@@ -32425,7 +32425,7 @@
         </is>
       </c>
       <c r="D1146" s="2" t="n">
-        <v>743</v>
+        <v>719</v>
       </c>
       <c r="E1146" s="3" t="n">
         <v>6111</v>
@@ -32761,7 +32761,7 @@
         </is>
       </c>
       <c r="D1158" s="2" t="n">
-        <v>249</v>
+        <v>225</v>
       </c>
       <c r="E1158" s="3" t="n">
         <v>9174</v>
@@ -33013,7 +33013,7 @@
         </is>
       </c>
       <c r="D1167" s="2" t="n">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E1167" s="3" t="n">
         <v>13001</v>
@@ -34161,7 +34161,7 @@
         </is>
       </c>
       <c r="D1208" s="2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E1208" s="3" t="n">
         <v>24420</v>
@@ -35449,7 +35449,7 @@
         </is>
       </c>
       <c r="D1254" s="2" t="n">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E1254" s="3" t="n">
         <v>3391</v>
@@ -35533,7 +35533,7 @@
         </is>
       </c>
       <c r="D1257" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E1257" s="3" t="n">
         <v>36976</v>
@@ -35953,7 +35953,7 @@
         </is>
       </c>
       <c r="D1272" s="2" t="n">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="E1272" s="3" t="n">
         <v>10600</v>
@@ -36793,7 +36793,7 @@
         </is>
       </c>
       <c r="D1302" s="2" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E1302" s="3" t="n">
         <v>11774</v>
@@ -38445,7 +38445,7 @@
         </is>
       </c>
       <c r="D1361" s="2" t="n">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="E1361" s="3" t="n">
         <v>8318</v>
@@ -39873,7 +39873,7 @@
         </is>
       </c>
       <c r="D1412" s="2" t="n">
-        <v>192</v>
+        <v>156</v>
       </c>
       <c r="E1412" s="3" t="n">
         <v>9036</v>
@@ -39901,7 +39901,7 @@
         </is>
       </c>
       <c r="D1413" s="2" t="n">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="E1413" s="3" t="n">
         <v>8626</v>
@@ -40293,7 +40293,7 @@
         </is>
       </c>
       <c r="D1427" s="2" t="n">
-        <v>1006</v>
+        <v>1000</v>
       </c>
       <c r="E1427" s="3" t="n">
         <v>5519</v>
@@ -40349,7 +40349,7 @@
         </is>
       </c>
       <c r="D1429" s="2" t="n">
-        <v>766</v>
+        <v>754</v>
       </c>
       <c r="E1429" s="3" t="n">
         <v>3140</v>
@@ -40657,7 +40657,7 @@
         </is>
       </c>
       <c r="D1440" s="2" t="n">
-        <v>6</v>
+        <v>-6</v>
       </c>
       <c r="E1440" s="3" t="n">
         <v>10733</v>
@@ -41581,7 +41581,7 @@
         </is>
       </c>
       <c r="D1473" s="2" t="n">
-        <v>2530</v>
+        <v>2506</v>
       </c>
       <c r="E1473" s="3" t="n">
         <v>7312</v>
@@ -41637,7 +41637,7 @@
         </is>
       </c>
       <c r="D1475" s="2" t="n">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="E1475" s="3" t="n">
         <v>10267</v>
@@ -41805,7 +41805,7 @@
         </is>
       </c>
       <c r="D1481" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E1481" s="3" t="n">
         <v>12610</v>
@@ -42029,7 +42029,7 @@
         </is>
       </c>
       <c r="D1489" s="2" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E1489" s="3" t="n">
         <v>7781</v>
@@ -42253,7 +42253,7 @@
         </is>
       </c>
       <c r="D1497" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E1497" s="3" t="n">
         <v>37512</v>
@@ -42421,7 +42421,7 @@
         </is>
       </c>
       <c r="D1503" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E1503" s="3" t="n">
         <v>12491</v>
@@ -43206,7 +43206,7 @@
         </is>
       </c>
       <c r="D1531" s="2" t="n">
-        <v>265</v>
+        <v>241</v>
       </c>
       <c r="E1531" s="3" t="n">
         <v>23146</v>
@@ -43991,7 +43991,7 @@
         </is>
       </c>
       <c r="D1559" s="2" t="n">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="E1559" s="3" t="n">
         <v>10097</v>

</xml_diff>